<commit_message>
Narayen APSIM Annual summary 1970 - 1990
</commit_message>
<xml_diff>
--- a/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedLWG.xlsx
+++ b/Tests/Validation/System/NarayenLongTermGrazingTrial/ObservedLWG.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Verson control in Git\ApsimX\Tests\Validation\System\NarayenLongTermGrazingTrial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE8F4BF-A667-48A6-A338-CA1A4EA6EE8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E5F23C-6A9D-4B68-A6DB-8C87AC0A3513}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="11829" activeTab="1" xr2:uid="{D13FB94D-EA64-45DA-AB49-15A51A1E985B}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D13FB94D-EA64-45DA-AB49-15A51A1E985B}"/>
   </bookViews>
   <sheets>
     <sheet name="Observed" sheetId="1" r:id="rId1"/>
@@ -1197,6 +1197,7 @@
   <cols>
     <col min="1" max="1" width="23.53515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.69140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.4">

</xml_diff>